<commit_message>
Push changes from current machine
</commit_message>
<xml_diff>
--- a/Check_Registered/Data/Documents/Config.xlsx
+++ b/Check_Registered/Data/Documents/Config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UiPathProjects\UiPathAutomation\Check_Registered\Data\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DeokateLaxman\Documents\UiPathAutomation\Check_Registered\Data\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F51DE7A-0708-46B8-A2B6-C78945D34CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C83DCEF-5AB9-4BDE-897F-A2229B94095B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -51,9 +51,6 @@
     <t>Downloads</t>
   </si>
   <si>
-    <t>C:\Users\laxma\Downloads</t>
-  </si>
-  <si>
     <t>https://efilingigr.maharashtra.gov.in/ereg/frmPoliceVerification.aspx</t>
   </si>
   <si>
@@ -354,7 +351,10 @@
     <t>Description (Assets will always overwrite other config)</t>
   </si>
   <si>
-    <t>D:\UiPathProjects\UiPathAutomation\Check_Registered\Data\Documents</t>
+    <t>C:\Users\DeokateLaxman\Documents\UiPathAutomation\Check_Registered\Data\Documents</t>
+  </si>
+  <si>
+    <t>C:\Users\DeokateLaxman\Downloads</t>
   </si>
 </sst>
 </file>
@@ -704,12 +704,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z993"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="43.5703125" customWidth="1"/>
-    <col min="2" max="2" width="95.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="81.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="1" max="1" width="43.54296875" customWidth="1"/>
+    <col min="2" max="2" width="95.1796875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="81.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -746,7 +746,7 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" s="4" customFormat="1" ht="15.75">
+    <row r="2" spans="1:26" s="4" customFormat="1" ht="15.5">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -754,7 +754,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="18.75">
+    <row r="3" spans="1:26" ht="18.5">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -791,7 +791,7 @@
         <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
@@ -799,164 +799,164 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>9</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>23</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18" t="s">
         <v>33</v>
-      </c>
-      <c r="B18" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
+        <v>40</v>
+      </c>
+      <c r="B23" t="s">
         <v>41</v>
-      </c>
-      <c r="B23" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" t="s">
+        <v>44</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="27" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28" s="2">
         <v>9011092282</v>
@@ -964,33 +964,33 @@
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
+        <v>47</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B34" s="2">
         <v>1000</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="35" spans="1:3" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B35" s="2">
         <v>300</v>
@@ -1006,66 +1006,66 @@
     </row>
     <row r="36" spans="1:3" ht="14.25" customHeight="1">
       <c r="A36" t="s">
+        <v>55</v>
+      </c>
+      <c r="B36" t="s">
         <v>56</v>
-      </c>
-      <c r="B36" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="14.25" customHeight="1">
       <c r="A37" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="39" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="40" spans="1:3" ht="14.25" customHeight="1">
       <c r="B40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="42" spans="1:3" ht="14.25" customHeight="1">
       <c r="A42" t="s">
+        <v>60</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="C42" t="s">
         <v>62</v>
-      </c>
-      <c r="C42" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="14.25" customHeight="1">
       <c r="A43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B43" s="7"/>
       <c r="C43" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="14.25" customHeight="1"/>
     <row r="45" spans="1:3" ht="14.25" customHeight="1">
       <c r="A45" t="s">
+        <v>65</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B45" s="2" t="s">
+      <c r="C45" t="s">
         <v>67</v>
-      </c>
-      <c r="C45" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="14.25" customHeight="1">
       <c r="A46" t="s">
+        <v>68</v>
+      </c>
+      <c r="B46" t="s">
         <v>69</v>
-      </c>
-      <c r="B46" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="14.25" customHeight="1"/>
@@ -2024,12 +2024,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z988"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="41" customWidth="1"/>
     <col min="2" max="2" width="51" customWidth="1"/>
-    <col min="3" max="3" width="75.42578125" customWidth="1"/>
-    <col min="4" max="26" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="75.453125" customWidth="1"/>
+    <col min="4" max="26" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -2066,145 +2066,145 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="30">
+    <row r="2" spans="1:26" ht="29">
       <c r="A2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="43.5">
+      <c r="A3" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" ht="45">
-      <c r="A3" t="s">
-        <v>73</v>
       </c>
       <c r="B3">
         <v>20</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
       <c r="A5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" t="s">
         <v>75</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>76</v>
-      </c>
-      <c r="C5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" t="s">
         <v>78</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>79</v>
-      </c>
-      <c r="C7" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1">
       <c r="A8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" t="s">
         <v>81</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>82</v>
-      </c>
-      <c r="C8" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" t="s">
         <v>84</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>85</v>
-      </c>
-      <c r="C9" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" t="s">
+        <v>86</v>
+      </c>
+      <c r="B10" t="s">
         <v>87</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>88</v>
-      </c>
-      <c r="C10" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" t="s">
+        <v>89</v>
+      </c>
+      <c r="B11" t="s">
         <v>90</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>91</v>
-      </c>
-      <c r="C11" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
       <c r="A12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
         <v>93</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>94</v>
-      </c>
-      <c r="C12" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B14">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B15">
         <v>2</v>
       </c>
       <c r="C15" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="17" spans="1:3" ht="29">
+      <c r="A17" t="s">
         <v>99</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="17" spans="1:3" ht="45">
-      <c r="A17" t="s">
-        <v>100</v>
       </c>
       <c r="B17" t="b">
         <v>0</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B18">
         <v>5</v>
@@ -2212,7 +2212,7 @@
     </row>
     <row r="19" spans="1:3" ht="14.25" customHeight="1">
       <c r="A19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B19">
         <v>5</v>
@@ -2220,7 +2220,7 @@
     </row>
     <row r="20" spans="1:3" ht="14.25" customHeight="1">
       <c r="A20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B20">
         <v>1.5</v>
@@ -2228,7 +2228,7 @@
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
       <c r="A21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B21">
         <v>1</v>
@@ -2236,7 +2236,7 @@
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
       <c r="A22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B22">
         <v>3</v>
@@ -3216,12 +3216,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.140625" customWidth="1"/>
-    <col min="3" max="3" width="60.28515625" customWidth="1"/>
-    <col min="4" max="26" width="65.42578125" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
+    <col min="2" max="2" width="30.1796875" customWidth="1"/>
+    <col min="3" max="3" width="60.26953125" customWidth="1"/>
+    <col min="4" max="26" width="65.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
@@ -3229,13 +3229,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>

</xml_diff>